<commit_message>
V4: Add TF_Sector and TF_Classification columns from Equity_Master.xlsx to both portfolio sheets
</commit_message>
<xml_diff>
--- a/Transformed_Tradebook.xlsx
+++ b/Transformed_Tradebook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/143b6e31b9e74e02/Desktop/Projects/stockjournal/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_28C34E415CEA97DD4F394E7496E91191A07EBC32" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC48A90F-05EC-4098-83A6-E159AB3B9B60}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="11_AA78CF5F257A5AA813B84D7496E91191C0FEF95A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E54A671-1C06-44B9-8AD3-AE781D2692B1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Raw_Tradebook" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3194" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3196" uniqueCount="327">
   <si>
     <t>Unnamed: 0.1</t>
   </si>
@@ -968,6 +968,9 @@
   </si>
   <si>
     <t>Unrealized_PnL</t>
+  </si>
+  <si>
+    <t>Holding_Period</t>
   </si>
   <si>
     <t>Mid Cap</t>
@@ -1349,8 +1352,20 @@
   <dimension ref="A1:O306"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="12" max="12" width="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="12" width="10" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -16667,7 +16682,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -16680,10 +16695,10 @@
     <col min="8" max="9" width="15" bestFit="1" customWidth="1"/>
     <col min="10" max="14" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="14" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="17" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -16732,13 +16747,16 @@
       <c r="P1" t="s">
         <v>314</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q1" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>201</v>
       </c>
       <c r="B2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C2" t="s">
         <v>293</v>
@@ -16782,13 +16800,16 @@
       <c r="P2" s="1">
         <v>222.8</v>
       </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>254</v>
       </c>
       <c r="B3" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C3" t="s">
         <v>292</v>
@@ -16832,13 +16853,16 @@
       <c r="P3" s="1">
         <v>-3816</v>
       </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>139</v>
       </c>
       <c r="B4" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C4" t="s">
         <v>292</v>
@@ -16882,13 +16906,16 @@
       <c r="P4" s="1">
         <v>292.5</v>
       </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q4">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>217</v>
       </c>
       <c r="B5" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C5" t="s">
         <v>294</v>
@@ -16932,13 +16959,16 @@
       <c r="P5" s="1">
         <v>-976.5</v>
       </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q5">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>236</v>
       </c>
       <c r="B6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C6" t="s">
         <v>292</v>
@@ -16982,13 +17012,16 @@
       <c r="P6" s="1">
         <v>3216.78</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q6">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>130</v>
       </c>
       <c r="B7" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C7" t="s">
         <v>293</v>
@@ -17032,13 +17065,16 @@
       <c r="P7" s="1">
         <v>-1225.9000000000001</v>
       </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q7">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>78</v>
       </c>
       <c r="B8" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C8" t="s">
         <v>293</v>
@@ -17082,13 +17118,16 @@
       <c r="P8" s="1">
         <v>-900</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q8">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C9" t="s">
         <v>296</v>
@@ -17132,13 +17171,16 @@
       <c r="P9" s="1">
         <v>-1045.25</v>
       </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q9">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>193</v>
       </c>
       <c r="B10" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C10" t="s">
         <v>296</v>
@@ -17182,13 +17224,16 @@
       <c r="P10" s="1">
         <v>-70388.800000000003</v>
       </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q10">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>142</v>
       </c>
       <c r="B11" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C11" t="s">
         <v>299</v>
@@ -17232,13 +17277,16 @@
       <c r="P11" s="1">
         <v>35488.160000000003</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q11">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>190</v>
       </c>
       <c r="B12" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C12" t="s">
         <v>294</v>
@@ -17282,13 +17330,16 @@
       <c r="P12" s="1">
         <v>-1086</v>
       </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q12">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>44</v>
       </c>
       <c r="B13" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C13" t="s">
         <v>296</v>
@@ -17332,13 +17383,16 @@
       <c r="P13" s="1">
         <v>-1764.64</v>
       </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q13">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>118</v>
       </c>
       <c r="B14" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C14" t="s">
         <v>294</v>
@@ -17382,13 +17436,16 @@
       <c r="P14" s="1">
         <v>-8663.64</v>
       </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q14">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>25</v>
       </c>
       <c r="B15" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C15" t="s">
         <v>297</v>
@@ -17432,13 +17489,16 @@
       <c r="P15" s="1">
         <v>-45543.519999999997</v>
       </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q15">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>88</v>
       </c>
       <c r="B16" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C16" t="s">
         <v>299</v>
@@ -17482,13 +17542,16 @@
       <c r="P16" s="1">
         <v>29244.27</v>
       </c>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q16">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>123</v>
       </c>
       <c r="B17" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C17" t="s">
         <v>292</v>
@@ -17532,13 +17595,16 @@
       <c r="P17" s="1">
         <v>-16072</v>
       </c>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q17">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>133</v>
       </c>
       <c r="B18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C18" t="s">
         <v>294</v>
@@ -17582,13 +17648,16 @@
       <c r="P18" s="1">
         <v>-5075.8999999999996</v>
       </c>
-    </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q18">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>220</v>
       </c>
       <c r="B19" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C19" t="s">
         <v>296</v>
@@ -17632,13 +17701,16 @@
       <c r="P19" s="1">
         <v>-403.2</v>
       </c>
-    </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q19">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>285</v>
       </c>
       <c r="B20" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C20" t="s">
         <v>293</v>
@@ -17682,13 +17754,16 @@
       <c r="P20" s="1">
         <v>-6.05</v>
       </c>
-    </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q20">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>187</v>
       </c>
       <c r="B21" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C21" t="s">
         <v>293</v>
@@ -17732,13 +17807,16 @@
       <c r="P21" s="1">
         <v>-1410</v>
       </c>
-    </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q21">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C22" t="s">
         <v>299</v>
@@ -17782,13 +17860,16 @@
       <c r="P22" s="1">
         <v>37295.1</v>
       </c>
-    </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q22">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>81</v>
       </c>
       <c r="B23" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C23" t="s">
         <v>292</v>
@@ -17832,13 +17913,16 @@
       <c r="P23" s="1">
         <v>-2696</v>
       </c>
-    </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q23">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>136</v>
       </c>
       <c r="B24" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C24" t="s">
         <v>297</v>
@@ -17882,13 +17966,16 @@
       <c r="P24" s="1">
         <v>4374.24</v>
       </c>
-    </row>
-    <row r="25" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q24">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>239</v>
       </c>
       <c r="B25" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C25" t="s">
         <v>296</v>
@@ -17932,13 +18019,16 @@
       <c r="P25" s="1">
         <v>-69.02</v>
       </c>
-    </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q25">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>273</v>
       </c>
       <c r="B26" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C26" t="s">
         <v>293</v>
@@ -17982,13 +18072,16 @@
       <c r="P26" s="1">
         <v>-1684</v>
       </c>
-    </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q26">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>258</v>
       </c>
       <c r="B27" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C27" t="s">
         <v>294</v>
@@ -18032,13 +18125,16 @@
       <c r="P27" s="1">
         <v>-1067</v>
       </c>
-    </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="Q27">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>47</v>
       </c>
       <c r="B28" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C28" t="s">
         <v>293</v>
@@ -18081,6 +18177,9 @@
       </c>
       <c r="P28" s="1">
         <v>-6212.3</v>
+      </c>
+      <c r="Q28">
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -18090,7 +18189,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:Q51"/>
+  <dimension ref="A1:R51"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -18110,9 +18209,10 @@
     <col min="15" max="15" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="11.42578125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -18123,22 +18223,22 @@
         <v>301</v>
       </c>
       <c r="D1" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="E1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="F1" t="s">
         <v>303</v>
       </c>
       <c r="G1" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="H1" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="I1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="J1" t="s">
         <v>302</v>
@@ -18153,24 +18253,27 @@
         <v>313</v>
       </c>
       <c r="N1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="O1" t="s">
         <v>314</v>
       </c>
       <c r="P1" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="Q1" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+        <v>326</v>
+      </c>
+      <c r="R1" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>201</v>
       </c>
       <c r="B2" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C2" t="s">
         <v>293</v>
@@ -18217,13 +18320,16 @@
       <c r="Q2" s="2">
         <v>1.896945135033886E-2</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>254</v>
       </c>
       <c r="B3" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C3" t="s">
         <v>292</v>
@@ -18270,13 +18376,16 @@
       <c r="Q3" s="2">
         <v>-3.7897745893021723E-2</v>
       </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>40</v>
       </c>
       <c r="B4" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C4" t="s">
         <v>298</v>
@@ -18323,13 +18432,16 @@
       <c r="Q4" s="2">
         <v>-7.2121731666699815E-2</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R4">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>98</v>
       </c>
       <c r="B5" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C5" t="s">
         <v>292</v>
@@ -18376,13 +18488,16 @@
       <c r="Q5" s="2">
         <v>-0.15634980274281421</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R5">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>139</v>
       </c>
       <c r="B6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C6" t="s">
         <v>292</v>
@@ -18429,13 +18544,16 @@
       <c r="Q6" s="2">
         <v>-4.2127959339530723E-2</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R6">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>217</v>
       </c>
       <c r="B7" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C7" t="s">
         <v>294</v>
@@ -18482,13 +18600,16 @@
       <c r="Q7" s="2">
         <v>-1.2988925295123939E-2</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R7">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>236</v>
       </c>
       <c r="B8" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C8" t="s">
         <v>292</v>
@@ -18535,13 +18656,16 @@
       <c r="Q8" s="2">
         <v>3.1919387367810019E-2</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R8">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>154</v>
       </c>
       <c r="B9" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C9" t="s">
         <v>293</v>
@@ -18588,13 +18712,16 @@
       <c r="Q9" s="2">
         <v>1.635815755488592E-2</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R9">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>130</v>
       </c>
       <c r="B10" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C10" t="s">
         <v>293</v>
@@ -18641,13 +18768,16 @@
       <c r="Q10" s="2">
         <v>-4.0658145227087307E-2</v>
       </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R10">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>78</v>
       </c>
       <c r="B11" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C11" t="s">
         <v>293</v>
@@ -18694,13 +18824,16 @@
       <c r="Q11" s="2">
         <v>-1.784694396605711E-2</v>
       </c>
-    </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R11">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>168</v>
       </c>
       <c r="B12" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C12" t="s">
         <v>294</v>
@@ -18747,13 +18880,16 @@
       <c r="Q12" s="2">
         <v>-9.7650586039835993E-2</v>
       </c>
-    </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R12">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>61</v>
       </c>
       <c r="B13" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C13" t="s">
         <v>297</v>
@@ -18800,13 +18936,16 @@
       <c r="Q13" s="2">
         <v>-1.5179777329596531E-2</v>
       </c>
-    </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R13">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>53</v>
       </c>
       <c r="B14" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C14" t="s">
         <v>296</v>
@@ -18853,13 +18992,16 @@
       <c r="Q14" s="2">
         <v>-1.126705641788092E-2</v>
       </c>
-    </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R14">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>127</v>
       </c>
       <c r="B15" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C15" t="s">
         <v>293</v>
@@ -18906,13 +19048,16 @@
       <c r="Q15" s="2">
         <v>-0.19539816748677671</v>
       </c>
-    </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R15">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>22</v>
       </c>
       <c r="B16" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C16" t="s">
         <v>292</v>
@@ -18959,13 +19104,16 @@
       <c r="Q16" s="2">
         <v>-0.16108205823487631</v>
       </c>
-    </row>
-    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R16">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>193</v>
       </c>
       <c r="B17" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C17" t="s">
         <v>296</v>
@@ -19012,13 +19160,16 @@
       <c r="Q17" s="2">
         <v>-0.54607109448082325</v>
       </c>
-    </row>
-    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R17">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>34</v>
       </c>
       <c r="B18" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C18" t="s">
         <v>292</v>
@@ -19065,13 +19216,16 @@
       <c r="Q18" s="2">
         <v>-0.14124164590966029</v>
       </c>
-    </row>
-    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R18">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>108</v>
       </c>
       <c r="B19" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C19" t="s">
         <v>293</v>
@@ -19118,13 +19272,16 @@
       <c r="Q19" s="2">
         <v>-0.1015625</v>
       </c>
-    </row>
-    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R19">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>142</v>
       </c>
       <c r="B20" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C20" t="s">
         <v>299</v>
@@ -19171,13 +19328,16 @@
       <c r="Q20" s="2">
         <v>0.1181814839541918</v>
       </c>
-    </row>
-    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R20">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>190</v>
       </c>
       <c r="B21" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C21" t="s">
         <v>294</v>
@@ -19224,13 +19384,16 @@
       <c r="Q21" s="2">
         <v>-2.1620851101020942E-2</v>
       </c>
-    </row>
-    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R21">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>44</v>
       </c>
       <c r="B22" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C22" t="s">
         <v>296</v>
@@ -19277,13 +19440,16 @@
       <c r="Q22" s="2">
         <v>-8.7397888650716238E-3</v>
       </c>
-    </row>
-    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R22">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>165</v>
       </c>
       <c r="B23" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C23" t="s">
         <v>292</v>
@@ -19330,13 +19496,16 @@
       <c r="Q23" s="2">
         <v>-0.17265855457227139</v>
       </c>
-    </row>
-    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R23">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>118</v>
       </c>
       <c r="B24" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C24" t="s">
         <v>294</v>
@@ -19383,13 +19552,16 @@
       <c r="Q24" s="2">
         <v>-0.1126134809293286</v>
       </c>
-    </row>
-    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R24">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>25</v>
       </c>
       <c r="B25" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C25" t="s">
         <v>297</v>
@@ -19436,13 +19608,16 @@
       <c r="Q25" s="2">
         <v>-0.2294130773481414</v>
       </c>
-    </row>
-    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R25">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>88</v>
       </c>
       <c r="B26" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C26" t="s">
         <v>299</v>
@@ -19489,13 +19664,16 @@
       <c r="Q26" s="2">
         <v>0.14022313022513869</v>
       </c>
-    </row>
-    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R26">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>123</v>
       </c>
       <c r="B27" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C27" t="s">
         <v>292</v>
@@ -19542,13 +19720,16 @@
       <c r="Q27" s="2">
         <v>-0.16220130340333089</v>
       </c>
-    </row>
-    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R27">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>133</v>
       </c>
       <c r="B28" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C28" t="s">
         <v>294</v>
@@ -19595,13 +19776,16 @@
       <c r="Q28" s="2">
         <v>-7.2320381612935844E-2</v>
       </c>
-    </row>
-    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R28">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>57</v>
       </c>
       <c r="B29" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C29" t="s">
         <v>293</v>
@@ -19648,13 +19832,16 @@
       <c r="Q29" s="2">
         <v>-9.7171155551569868E-2</v>
       </c>
-    </row>
-    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R29">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>174</v>
       </c>
       <c r="B30" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C30" t="s">
         <v>294</v>
@@ -19701,13 +19888,16 @@
       <c r="Q30" s="2">
         <v>-0.17667114643858131</v>
       </c>
-    </row>
-    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R30">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>179</v>
       </c>
       <c r="B31" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C31" t="s">
         <v>293</v>
@@ -19754,13 +19944,16 @@
       <c r="Q31" s="2">
         <v>-0.14019473604138141</v>
       </c>
-    </row>
-    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R31">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>220</v>
       </c>
       <c r="B32" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C32" t="s">
         <v>296</v>
@@ -19807,13 +20000,16 @@
       <c r="Q32" s="2">
         <v>-7.9214627829756919E-3</v>
       </c>
-    </row>
-    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R32">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>37</v>
       </c>
       <c r="B33" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C33" t="s">
         <v>292</v>
@@ -19860,13 +20056,16 @@
       <c r="Q33" s="2">
         <v>-0.1109521617118302</v>
       </c>
-    </row>
-    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R33">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>285</v>
       </c>
       <c r="B34" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C34" t="s">
         <v>293</v>
@@ -19913,13 +20112,16 @@
       <c r="Q34" s="2">
         <v>-2.4201355275895451E-4</v>
       </c>
-    </row>
-    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>187</v>
       </c>
       <c r="B35" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C35" t="s">
         <v>293</v>
@@ -19966,13 +20168,16 @@
       <c r="Q35" s="2">
         <v>-5.5627884956799621E-2</v>
       </c>
-    </row>
-    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R35">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>50</v>
       </c>
       <c r="B36" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C36" t="s">
         <v>292</v>
@@ -20019,13 +20224,16 @@
       <c r="Q36" s="2">
         <v>-0.51718403311145245</v>
       </c>
-    </row>
-    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R36">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>214</v>
       </c>
       <c r="B37" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C37" t="s">
         <v>294</v>
@@ -20072,13 +20280,16 @@
       <c r="Q37" s="2">
         <v>-6.3742898422480723E-2</v>
       </c>
-    </row>
-    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R37">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>15</v>
       </c>
       <c r="B38" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C38" t="s">
         <v>299</v>
@@ -20125,13 +20336,16 @@
       <c r="Q38" s="2">
         <v>0.12964046982595301</v>
       </c>
-    </row>
-    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R38">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>81</v>
       </c>
       <c r="B39" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C39" t="s">
         <v>292</v>
@@ -20178,13 +20392,16 @@
       <c r="Q39" s="2">
         <v>-0.10748007986573591</v>
       </c>
-    </row>
-    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R39">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>84</v>
       </c>
       <c r="B40" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C40" t="s">
         <v>294</v>
@@ -20231,13 +20448,16 @@
       <c r="Q40" s="2">
         <v>9.7625625824357127E-5</v>
       </c>
-    </row>
-    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R40">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="41" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>263</v>
       </c>
       <c r="B41" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C41" t="s">
         <v>293</v>
@@ -20284,13 +20504,16 @@
       <c r="Q41" s="2">
         <v>-0.1328714714093682</v>
       </c>
-    </row>
-    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R41">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>136</v>
       </c>
       <c r="B42" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C42" t="s">
         <v>297</v>
@@ -20337,13 +20560,16 @@
       <c r="Q42" s="2">
         <v>1.874380543506253E-2</v>
       </c>
-    </row>
-    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R42">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>239</v>
       </c>
       <c r="B43" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C43" t="s">
         <v>296</v>
@@ -20390,13 +20616,16 @@
       <c r="Q43" s="2">
         <v>-1.5059051467395689E-3</v>
       </c>
-    </row>
-    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R43">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="44" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>211</v>
       </c>
       <c r="B44" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C44" t="s">
         <v>293</v>
@@ -20443,13 +20672,16 @@
       <c r="Q44" s="2">
         <v>-0.1555351922644479</v>
       </c>
-    </row>
-    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R44">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="45" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>67</v>
       </c>
       <c r="B45" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C45" t="s">
         <v>293</v>
@@ -20496,13 +20728,16 @@
       <c r="Q45" s="2">
         <v>-0.10584928229665071</v>
       </c>
-    </row>
-    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R45">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>28</v>
       </c>
       <c r="B46" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C46" t="s">
         <v>292</v>
@@ -20549,13 +20784,16 @@
       <c r="Q46" s="2">
         <v>-7.2933022843202494E-2</v>
       </c>
-    </row>
-    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R46">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>273</v>
       </c>
       <c r="B47" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C47" t="s">
         <v>293</v>
@@ -20602,13 +20840,16 @@
       <c r="Q47" s="2">
         <v>-6.688915386809173E-2</v>
       </c>
-    </row>
-    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R47">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="48" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>258</v>
       </c>
       <c r="B48" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C48" t="s">
         <v>294</v>
@@ -20655,13 +20896,16 @@
       <c r="Q48" s="2">
         <v>-2.1599846149174571E-2</v>
       </c>
-    </row>
-    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R48">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="49" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>31</v>
       </c>
       <c r="B49" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="C49" t="s">
         <v>292</v>
@@ -20708,13 +20952,16 @@
       <c r="Q49" s="2">
         <v>-7.431676085947525E-2</v>
       </c>
-    </row>
-    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R49">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="50" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>157</v>
       </c>
       <c r="B50" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="C50" t="s">
         <v>294</v>
@@ -20761,13 +21008,16 @@
       <c r="Q50" s="2">
         <v>-0.1262705760049663</v>
       </c>
-    </row>
-    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R50">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="51" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>47</v>
       </c>
       <c r="B51" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C51" t="s">
         <v>293</v>
@@ -20813,6 +21063,9 @@
       </c>
       <c r="Q51" s="2">
         <v>-0.13023580515048089</v>
+      </c>
+      <c r="R51">
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add Previous Day Closing Price column to Current Portfolio next to LTP
</commit_message>
<xml_diff>
--- a/Transformed_Tradebook.xlsx
+++ b/Transformed_Tradebook.xlsx
@@ -32512,7 +32512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V30"/>
+  <dimension ref="A1:W30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="27" min="1" max="1"/>
@@ -32527,16 +32527,17 @@
     <col width="27" customWidth="1" style="27" min="10" max="10"/>
     <col width="16" customWidth="1" style="27" min="11" max="11"/>
     <col width="14" customWidth="1" style="27" min="12" max="12"/>
-    <col width="17" customWidth="1" style="27" min="13" max="13"/>
-    <col width="15" customWidth="1" style="27" min="14" max="14"/>
+    <col width="16" customWidth="1" style="27" min="13" max="13"/>
+    <col width="17" customWidth="1" style="27" min="14" max="14"/>
     <col width="15" customWidth="1" style="27" min="15" max="15"/>
-    <col width="14" customWidth="1" style="27" min="16" max="16"/>
-    <col width="15" customWidth="1" style="27" min="17" max="17"/>
-    <col width="16" customWidth="1" style="27" min="18" max="18"/>
+    <col width="15" customWidth="1" style="27" min="16" max="16"/>
+    <col width="14" customWidth="1" style="27" min="17" max="17"/>
+    <col width="15" customWidth="1" style="27" min="18" max="18"/>
     <col width="16" customWidth="1" style="27" min="19" max="19"/>
     <col width="16" customWidth="1" style="27" min="20" max="20"/>
-    <col width="25" customWidth="1" style="27" min="21" max="21"/>
-    <col width="14" customWidth="1" style="27" min="22" max="22"/>
+    <col width="16" customWidth="1" style="27" min="21" max="21"/>
+    <col width="25" customWidth="1" style="27" min="22" max="22"/>
+    <col width="14" customWidth="1" style="27" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -32602,50 +32603,55 @@
       </c>
       <c r="M1" s="48" t="inlineStr">
         <is>
+          <t>Prev_Day_Close</t>
+        </is>
+      </c>
+      <c r="N1" s="48" t="inlineStr">
+        <is>
           <t>Prev_Week_Close</t>
         </is>
       </c>
-      <c r="N1" s="48" t="inlineStr">
+      <c r="O1" s="48" t="inlineStr">
         <is>
           <t>EMA9</t>
         </is>
       </c>
-      <c r="O1" s="48" t="inlineStr">
+      <c r="P1" s="48" t="inlineStr">
         <is>
           <t>EMA10</t>
         </is>
       </c>
-      <c r="P1" s="48" t="inlineStr">
+      <c r="Q1" s="48" t="inlineStr">
         <is>
           <t>EMA11</t>
         </is>
       </c>
-      <c r="Q1" s="48" t="inlineStr">
+      <c r="R1" s="48" t="inlineStr">
         <is>
           <t>EMA21</t>
         </is>
       </c>
-      <c r="R1" s="48" t="inlineStr">
+      <c r="S1" s="48" t="inlineStr">
         <is>
           <t>Current_Value</t>
         </is>
       </c>
-      <c r="S1" s="48" t="inlineStr">
+      <c r="T1" s="48" t="inlineStr">
         <is>
           <t>Unrealized_PnL</t>
         </is>
       </c>
-      <c r="T1" s="48" t="inlineStr">
+      <c r="U1" s="48" t="inlineStr">
         <is>
           <t>Holding_Period</t>
         </is>
       </c>
-      <c r="U1" s="48" t="inlineStr">
+      <c r="V1" s="48" t="inlineStr">
         <is>
           <t>Split_Info</t>
         </is>
       </c>
-      <c r="V1" s="48" t="inlineStr">
+      <c r="W1" s="48" t="inlineStr">
         <is>
           <t>Adj_Required</t>
         </is>
@@ -32699,31 +32705,34 @@
         <v>2886.5</v>
       </c>
       <c r="M2" s="51" t="n">
+        <v>2799.1</v>
+      </c>
+      <c r="N2" s="51" t="n">
         <v>2731</v>
       </c>
-      <c r="N2" s="51" t="n">
+      <c r="O2" s="51" t="n">
         <v>2763.25</v>
       </c>
-      <c r="O2" s="51" t="n">
+      <c r="P2" s="51" t="n">
         <v>2752.93</v>
       </c>
-      <c r="P2" s="51" t="n">
+      <c r="Q2" s="51" t="n">
         <v>2742.62</v>
       </c>
-      <c r="Q2" s="51" t="n">
+      <c r="R2" s="51" t="n">
         <v>2648.69</v>
       </c>
-      <c r="R2" s="51" t="n">
+      <c r="S2" s="51" t="n">
         <v>51957</v>
       </c>
-      <c r="S2" s="51" t="n">
+      <c r="T2" s="51" t="n">
         <v>2817</v>
       </c>
-      <c r="T2" s="49" t="n">
+      <c r="U2" s="49" t="n">
         <v>4</v>
       </c>
-      <c r="U2" s="49" t="inlineStr"/>
-      <c r="V2" s="49" t="inlineStr">
+      <c r="V2" s="49" t="inlineStr"/>
+      <c r="W2" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -32777,31 +32786,34 @@
         <v>2725</v>
       </c>
       <c r="M3" s="51" t="n">
+        <v>2689.8</v>
+      </c>
+      <c r="N3" s="51" t="n">
         <v>2716</v>
       </c>
-      <c r="N3" s="51" t="n">
+      <c r="O3" s="51" t="n">
         <v>2404.44</v>
       </c>
-      <c r="O3" s="51" t="n">
+      <c r="P3" s="51" t="n">
         <v>2381.91</v>
       </c>
-      <c r="P3" s="51" t="n">
+      <c r="Q3" s="51" t="n">
         <v>2362.91</v>
       </c>
-      <c r="Q3" s="51" t="n">
+      <c r="R3" s="51" t="n">
         <v>2282.12</v>
       </c>
-      <c r="R3" s="51" t="n">
+      <c r="S3" s="51" t="n">
         <v>51775</v>
       </c>
-      <c r="S3" s="51" t="n">
+      <c r="T3" s="51" t="n">
         <v>-41.8</v>
       </c>
-      <c r="T3" s="49" t="n">
+      <c r="U3" s="49" t="n">
         <v>4</v>
       </c>
-      <c r="U3" s="49" t="inlineStr"/>
-      <c r="V3" s="49" t="inlineStr">
+      <c r="V3" s="49" t="inlineStr"/>
+      <c r="W3" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -32855,31 +32867,34 @@
         <v>3248.2</v>
       </c>
       <c r="M4" s="51" t="n">
+        <v>3214.1</v>
+      </c>
+      <c r="N4" s="51" t="n">
         <v>3177.2</v>
       </c>
-      <c r="N4" s="51" t="n">
+      <c r="O4" s="51" t="n">
         <v>2993.13</v>
       </c>
-      <c r="O4" s="51" t="n">
+      <c r="P4" s="51" t="n">
         <v>2980.46</v>
       </c>
-      <c r="P4" s="51" t="n">
+      <c r="Q4" s="51" t="n">
         <v>2969.06</v>
       </c>
-      <c r="Q4" s="51" t="n">
+      <c r="R4" s="51" t="n">
         <v>2885.09</v>
       </c>
-      <c r="R4" s="51" t="n">
+      <c r="S4" s="51" t="n">
         <v>45474.8</v>
       </c>
-      <c r="S4" s="51" t="n">
+      <c r="T4" s="51" t="n">
         <v>1589.56</v>
       </c>
-      <c r="T4" s="49" t="n">
+      <c r="U4" s="49" t="n">
         <v>134</v>
       </c>
-      <c r="U4" s="49" t="inlineStr"/>
-      <c r="V4" s="49" t="inlineStr">
+      <c r="V4" s="49" t="inlineStr"/>
+      <c r="W4" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -32933,31 +32948,34 @@
         <v>1864.5</v>
       </c>
       <c r="M5" s="51" t="n">
+        <v>1876</v>
+      </c>
+      <c r="N5" s="51" t="n">
         <v>1890.2</v>
       </c>
-      <c r="N5" s="51" t="n">
+      <c r="O5" s="51" t="n">
         <v>1896.42</v>
       </c>
-      <c r="O5" s="51" t="n">
+      <c r="P5" s="51" t="n">
         <v>1899.74</v>
       </c>
-      <c r="P5" s="51" t="n">
+      <c r="Q5" s="51" t="n">
         <v>1903</v>
       </c>
-      <c r="Q5" s="51" t="n">
+      <c r="R5" s="51" t="n">
         <v>1930.85</v>
       </c>
-      <c r="R5" s="51" t="n">
+      <c r="S5" s="51" t="n">
         <v>178992</v>
       </c>
-      <c r="S5" s="51" t="n">
+      <c r="T5" s="51" t="n">
         <v>-22684.8</v>
       </c>
-      <c r="T5" s="49" t="n">
+      <c r="U5" s="49" t="n">
         <v>99</v>
       </c>
-      <c r="U5" s="49" t="inlineStr"/>
-      <c r="V5" s="49" t="inlineStr">
+      <c r="V5" s="49" t="inlineStr"/>
+      <c r="W5" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -33011,31 +33029,34 @@
         <v>340.7</v>
       </c>
       <c r="M6" s="51" t="n">
+        <v>311</v>
+      </c>
+      <c r="N6" s="51" t="n">
         <v>294.55</v>
       </c>
-      <c r="N6" s="51" t="n">
+      <c r="O6" s="51" t="n">
         <v>286.26</v>
       </c>
-      <c r="O6" s="51" t="n">
+      <c r="P6" s="51" t="n">
         <v>282.74</v>
       </c>
-      <c r="P6" s="51" t="n">
+      <c r="Q6" s="51" t="n">
         <v>279.71</v>
       </c>
-      <c r="Q6" s="51" t="n">
+      <c r="R6" s="51" t="n">
         <v>263.78</v>
       </c>
-      <c r="R6" s="51" t="n">
+      <c r="S6" s="51" t="n">
         <v>58259.7</v>
       </c>
-      <c r="S6" s="51" t="n">
+      <c r="T6" s="51" t="n">
         <v>8011.35</v>
       </c>
-      <c r="T6" s="49" t="n">
+      <c r="U6" s="49" t="n">
         <v>15</v>
       </c>
-      <c r="U6" s="49" t="inlineStr"/>
-      <c r="V6" s="49" t="inlineStr">
+      <c r="V6" s="49" t="inlineStr"/>
+      <c r="W6" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -33089,31 +33110,34 @@
         <v>1092.7</v>
       </c>
       <c r="M7" s="51" t="n">
+        <v>1087.2</v>
+      </c>
+      <c r="N7" s="51" t="n">
         <v>1106.6</v>
       </c>
-      <c r="N7" s="51" t="n">
+      <c r="O7" s="51" t="n">
         <v>1071.35</v>
       </c>
-      <c r="O7" s="51" t="n">
+      <c r="P7" s="51" t="n">
         <v>1065.35</v>
       </c>
-      <c r="P7" s="51" t="n">
+      <c r="Q7" s="51" t="n">
         <v>1059.84</v>
       </c>
-      <c r="Q7" s="51" t="n">
+      <c r="R7" s="51" t="n">
         <v>1026.04</v>
       </c>
-      <c r="R7" s="51" t="n">
+      <c r="S7" s="51" t="n">
         <v>48078.8</v>
       </c>
-      <c r="S7" s="51" t="n">
+      <c r="T7" s="51" t="n">
         <v>-2149.4</v>
       </c>
-      <c r="T7" s="49" t="n">
+      <c r="U7" s="49" t="n">
         <v>22</v>
       </c>
-      <c r="U7" s="49" t="inlineStr"/>
-      <c r="V7" s="49" t="inlineStr">
+      <c r="V7" s="49" t="inlineStr"/>
+      <c r="W7" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -33167,31 +33191,34 @@
         <v>1512.8</v>
       </c>
       <c r="M8" s="51" t="n">
+        <v>1500.5</v>
+      </c>
+      <c r="N8" s="51" t="n">
         <v>1511.8</v>
       </c>
-      <c r="N8" s="51" t="n">
+      <c r="O8" s="51" t="n">
         <v>1419.55</v>
       </c>
-      <c r="O8" s="51" t="n">
+      <c r="P8" s="51" t="n">
         <v>1409.4</v>
       </c>
-      <c r="P8" s="51" t="n">
+      <c r="Q8" s="51" t="n">
         <v>1399.88</v>
       </c>
-      <c r="Q8" s="51" t="n">
+      <c r="R8" s="51" t="n">
         <v>1330.54</v>
       </c>
-      <c r="R8" s="51" t="n">
+      <c r="S8" s="51" t="n">
         <v>49922.4</v>
       </c>
-      <c r="S8" s="51" t="n">
+      <c r="T8" s="51" t="n">
         <v>237.6</v>
       </c>
-      <c r="T8" s="49" t="n">
+      <c r="U8" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="U8" s="49" t="inlineStr"/>
-      <c r="V8" s="49" t="inlineStr">
+      <c r="V8" s="49" t="inlineStr"/>
+      <c r="W8" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -33245,31 +33272,34 @@
         <v>1708.8</v>
       </c>
       <c r="M9" s="51" t="n">
+        <v>1763</v>
+      </c>
+      <c r="N9" s="51" t="n">
         <v>1706.2</v>
       </c>
-      <c r="N9" s="51" t="n">
+      <c r="O9" s="51" t="n">
         <v>1399.94</v>
       </c>
-      <c r="O9" s="51" t="n">
+      <c r="P9" s="51" t="n">
         <v>1379.1</v>
       </c>
-      <c r="P9" s="51" t="n">
+      <c r="Q9" s="51" t="n">
         <v>1361.36</v>
       </c>
-      <c r="Q9" s="51" t="n">
+      <c r="R9" s="51" t="n">
         <v>1282.54</v>
       </c>
-      <c r="R9" s="51" t="n">
+      <c r="S9" s="51" t="n">
         <v>49555.2</v>
       </c>
-      <c r="S9" s="51" t="n">
+      <c r="T9" s="51" t="n">
         <v>-133.98</v>
       </c>
-      <c r="T9" s="49" t="n">
+      <c r="U9" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="U9" s="49" t="inlineStr"/>
-      <c r="V9" s="49" t="inlineStr">
+      <c r="V9" s="49" t="inlineStr"/>
+      <c r="W9" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -33323,31 +33353,34 @@
         <v>4190.8</v>
       </c>
       <c r="M10" s="51" t="n">
+        <v>4120.7</v>
+      </c>
+      <c r="N10" s="51" t="n">
         <v>4000.6</v>
       </c>
-      <c r="N10" s="51" t="n">
+      <c r="O10" s="51" t="n">
         <v>3623.33</v>
       </c>
-      <c r="O10" s="51" t="n">
+      <c r="P10" s="51" t="n">
         <v>3575.74</v>
       </c>
-      <c r="P10" s="51" t="n">
+      <c r="Q10" s="51" t="n">
         <v>3532.3</v>
       </c>
-      <c r="Q10" s="51" t="n">
+      <c r="R10" s="51" t="n">
         <v>3236.77</v>
       </c>
-      <c r="R10" s="51" t="n">
+      <c r="S10" s="51" t="n">
         <v>75434.39999999999</v>
       </c>
-      <c r="S10" s="51" t="n">
+      <c r="T10" s="51" t="n">
         <v>25005.6</v>
       </c>
-      <c r="T10" s="49" t="n">
+      <c r="U10" s="49" t="n">
         <v>162</v>
       </c>
-      <c r="U10" s="49" t="inlineStr"/>
-      <c r="V10" s="49" t="inlineStr">
+      <c r="V10" s="49" t="inlineStr"/>
+      <c r="W10" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -33401,31 +33434,34 @@
         <v>1089.4</v>
       </c>
       <c r="M11" s="51" t="n">
+        <v>1090.4</v>
+      </c>
+      <c r="N11" s="51" t="n">
         <v>1116.3</v>
       </c>
-      <c r="N11" s="51" t="n">
+      <c r="O11" s="51" t="n">
         <v>1111.93</v>
       </c>
-      <c r="O11" s="51" t="n">
+      <c r="P11" s="51" t="n">
         <v>1113.34</v>
       </c>
-      <c r="P11" s="51" t="n">
+      <c r="Q11" s="51" t="n">
         <v>1114.44</v>
       </c>
-      <c r="Q11" s="51" t="n">
+      <c r="R11" s="51" t="n">
         <v>1115.26</v>
       </c>
-      <c r="R11" s="51" t="n">
+      <c r="S11" s="51" t="n">
         <v>53380.6</v>
       </c>
-      <c r="S11" s="51" t="n">
+      <c r="T11" s="51" t="n">
         <v>2755.76</v>
       </c>
-      <c r="T11" s="49" t="n">
+      <c r="U11" s="49" t="n">
         <v>71</v>
       </c>
-      <c r="U11" s="49" t="inlineStr"/>
-      <c r="V11" s="49" t="inlineStr">
+      <c r="V11" s="49" t="inlineStr"/>
+      <c r="W11" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -33479,31 +33515,34 @@
         <v>819.4</v>
       </c>
       <c r="M12" s="51" t="n">
+        <v>808.75</v>
+      </c>
+      <c r="N12" s="51" t="n">
         <v>838.2</v>
       </c>
-      <c r="N12" s="51" t="n">
+      <c r="O12" s="51" t="n">
         <v>792.23</v>
       </c>
-      <c r="O12" s="51" t="n">
+      <c r="P12" s="51" t="n">
         <v>786.23</v>
       </c>
-      <c r="P12" s="51" t="n">
+      <c r="Q12" s="51" t="n">
         <v>780.66</v>
       </c>
-      <c r="Q12" s="51" t="n">
+      <c r="R12" s="51" t="n">
         <v>744.23</v>
       </c>
-      <c r="R12" s="51" t="n">
+      <c r="S12" s="51" t="n">
         <v>77023.60000000001</v>
       </c>
-      <c r="S12" s="51" t="n">
+      <c r="T12" s="51" t="n">
         <v>1747.46</v>
       </c>
-      <c r="T12" s="49" t="n">
+      <c r="U12" s="49" t="n">
         <v>246</v>
       </c>
-      <c r="U12" s="49" t="inlineStr"/>
-      <c r="V12" s="49" t="inlineStr">
+      <c r="V12" s="49" t="inlineStr"/>
+      <c r="W12" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -33557,35 +33596,38 @@
         <v>114.34</v>
       </c>
       <c r="M13" s="51" t="n">
+        <v>120.84</v>
+      </c>
+      <c r="N13" s="51" t="n">
         <v>120.36</v>
       </c>
-      <c r="N13" s="51" t="n">
+      <c r="O13" s="51" t="n">
         <v>109.72</v>
       </c>
-      <c r="O13" s="51" t="n">
+      <c r="P13" s="51" t="n">
         <v>108.25</v>
       </c>
-      <c r="P13" s="51" t="n">
+      <c r="Q13" s="51" t="n">
         <v>106.86</v>
       </c>
-      <c r="Q13" s="51" t="n">
+      <c r="R13" s="51" t="n">
         <v>95.33</v>
       </c>
-      <c r="R13" s="51" t="n">
+      <c r="S13" s="51" t="n">
         <v>164192.24</v>
       </c>
-      <c r="S13" s="51" t="n">
+      <c r="T13" s="51" t="n">
         <v>32094.6</v>
       </c>
-      <c r="T13" s="49" t="n">
+      <c r="U13" s="49" t="n">
         <v>134</v>
       </c>
-      <c r="U13" s="49" t="inlineStr">
+      <c r="V13" s="49" t="inlineStr">
         <is>
           <t>5:1 Split on 2026-03-09</t>
         </is>
       </c>
-      <c r="V13" s="49" t="inlineStr">
+      <c r="W13" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -33639,31 +33681,34 @@
         <v>286.6</v>
       </c>
       <c r="M14" s="51" t="n">
+        <v>283.95</v>
+      </c>
+      <c r="N14" s="51" t="n">
         <v>281.3</v>
       </c>
-      <c r="N14" s="51" t="n">
+      <c r="O14" s="51" t="n">
         <v>285.62</v>
       </c>
-      <c r="O14" s="51" t="n">
+      <c r="P14" s="51" t="n">
         <v>285.13</v>
       </c>
-      <c r="P14" s="51" t="n">
+      <c r="Q14" s="51" t="n">
         <v>284.58</v>
       </c>
-      <c r="Q14" s="51" t="n">
+      <c r="R14" s="51" t="n">
         <v>276.81</v>
       </c>
-      <c r="R14" s="51" t="n">
+      <c r="S14" s="51" t="n">
         <v>335895.2</v>
       </c>
-      <c r="S14" s="51" t="n">
+      <c r="T14" s="51" t="n">
         <v>35605.36</v>
       </c>
-      <c r="T14" s="49" t="n">
+      <c r="U14" s="49" t="n">
         <v>197</v>
       </c>
-      <c r="U14" s="49" t="inlineStr"/>
-      <c r="V14" s="49" t="inlineStr">
+      <c r="V14" s="49" t="inlineStr"/>
+      <c r="W14" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -33717,31 +33762,34 @@
         <v>161.12</v>
       </c>
       <c r="M15" s="51" t="n">
+        <v>161.98</v>
+      </c>
+      <c r="N15" s="51" t="n">
         <v>162.79</v>
       </c>
-      <c r="N15" s="51" t="n">
+      <c r="O15" s="51" t="n">
         <v>154.07</v>
       </c>
-      <c r="O15" s="51" t="n">
+      <c r="P15" s="51" t="n">
         <v>153.01</v>
       </c>
-      <c r="P15" s="51" t="n">
+      <c r="Q15" s="51" t="n">
         <v>152</v>
       </c>
-      <c r="Q15" s="51" t="n">
+      <c r="R15" s="51" t="n">
         <v>143.69</v>
       </c>
-      <c r="R15" s="51" t="n">
+      <c r="S15" s="51" t="n">
         <v>58325.44</v>
       </c>
-      <c r="S15" s="51" t="n">
+      <c r="T15" s="51" t="n">
         <v>8097.94</v>
       </c>
-      <c r="T15" s="49" t="n">
+      <c r="U15" s="49" t="n">
         <v>137</v>
       </c>
-      <c r="U15" s="49" t="inlineStr"/>
-      <c r="V15" s="49" t="inlineStr">
+      <c r="V15" s="49" t="inlineStr"/>
+      <c r="W15" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -33795,31 +33843,34 @@
         <v>643.85</v>
       </c>
       <c r="M16" s="51" t="n">
+        <v>632.8</v>
+      </c>
+      <c r="N16" s="51" t="n">
         <v>652.6</v>
       </c>
-      <c r="N16" s="51" t="n">
+      <c r="O16" s="51" t="n">
         <v>649.59</v>
       </c>
-      <c r="O16" s="51" t="n">
+      <c r="P16" s="51" t="n">
         <v>646.04</v>
       </c>
-      <c r="P16" s="51" t="n">
+      <c r="Q16" s="51" t="n">
         <v>642.55</v>
       </c>
-      <c r="Q16" s="51" t="n">
+      <c r="R16" s="51" t="n">
         <v>612.38</v>
       </c>
-      <c r="R16" s="51" t="n">
+      <c r="S16" s="51" t="n">
         <v>26397.85</v>
       </c>
-      <c r="S16" s="51" t="n">
+      <c r="T16" s="51" t="n">
         <v>2212.36</v>
       </c>
-      <c r="T16" s="49" t="n">
+      <c r="U16" s="49" t="n">
         <v>252</v>
       </c>
-      <c r="U16" s="49" t="inlineStr"/>
-      <c r="V16" s="49" t="inlineStr">
+      <c r="V16" s="49" t="inlineStr"/>
+      <c r="W16" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -33873,31 +33924,34 @@
         <v>290.55</v>
       </c>
       <c r="M17" s="51" t="n">
+        <v>283.3</v>
+      </c>
+      <c r="N17" s="51" t="n">
         <v>287.9</v>
       </c>
-      <c r="N17" s="51" t="n">
+      <c r="O17" s="51" t="n">
         <v>286.24</v>
       </c>
-      <c r="O17" s="51" t="n">
+      <c r="P17" s="51" t="n">
         <v>285.06</v>
       </c>
-      <c r="P17" s="51" t="n">
+      <c r="Q17" s="51" t="n">
         <v>283.9</v>
       </c>
-      <c r="Q17" s="51" t="n">
+      <c r="R17" s="51" t="n">
         <v>273.59</v>
       </c>
-      <c r="R17" s="51" t="n">
+      <c r="S17" s="51" t="n">
         <v>80191.8</v>
       </c>
-      <c r="S17" s="51" t="n">
+      <c r="T17" s="51" t="n">
         <v>3259.56</v>
       </c>
-      <c r="T17" s="49" t="n">
+      <c r="U17" s="49" t="n">
         <v>204</v>
       </c>
-      <c r="U17" s="49" t="inlineStr"/>
-      <c r="V17" s="49" t="inlineStr">
+      <c r="V17" s="49" t="inlineStr"/>
+      <c r="W17" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -33951,31 +34005,34 @@
         <v>4385.3</v>
       </c>
       <c r="M18" s="51" t="n">
+        <v>4426.8</v>
+      </c>
+      <c r="N18" s="51" t="n">
         <v>4342.6</v>
       </c>
-      <c r="N18" s="51" t="n">
+      <c r="O18" s="51" t="n">
         <v>4410.37</v>
       </c>
-      <c r="O18" s="51" t="n">
+      <c r="P18" s="51" t="n">
         <v>4412.63</v>
       </c>
-      <c r="P18" s="51" t="n">
+      <c r="Q18" s="51" t="n">
         <v>4413.55</v>
       </c>
-      <c r="Q18" s="51" t="n">
+      <c r="R18" s="51" t="n">
         <v>4369.81</v>
       </c>
-      <c r="R18" s="51" t="n">
+      <c r="S18" s="51" t="n">
         <v>214879.7</v>
       </c>
-      <c r="S18" s="51" t="n">
+      <c r="T18" s="51" t="n">
         <v>14555.94</v>
       </c>
-      <c r="T18" s="49" t="n">
+      <c r="U18" s="49" t="n">
         <v>71</v>
       </c>
-      <c r="U18" s="49" t="inlineStr"/>
-      <c r="V18" s="49" t="inlineStr">
+      <c r="V18" s="49" t="inlineStr"/>
+      <c r="W18" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -34029,31 +34086,34 @@
         <v>1048.3</v>
       </c>
       <c r="M19" s="51" t="n">
+        <v>1053.1</v>
+      </c>
+      <c r="N19" s="51" t="n">
         <v>1067.5</v>
       </c>
-      <c r="N19" s="51" t="n">
+      <c r="O19" s="51" t="n">
         <v>1016.47</v>
       </c>
-      <c r="O19" s="51" t="n">
+      <c r="P19" s="51" t="n">
         <v>1010.99</v>
       </c>
-      <c r="P19" s="51" t="n">
+      <c r="Q19" s="51" t="n">
         <v>1005.73</v>
       </c>
-      <c r="Q19" s="51" t="n">
+      <c r="R19" s="51" t="n">
         <v>960.29</v>
       </c>
-      <c r="R19" s="51" t="n">
+      <c r="S19" s="51" t="n">
         <v>265219.9</v>
       </c>
-      <c r="S19" s="51" t="n">
+      <c r="T19" s="51" t="n">
         <v>51862.47</v>
       </c>
-      <c r="T19" s="49" t="n">
+      <c r="U19" s="49" t="n">
         <v>225</v>
       </c>
-      <c r="U19" s="49" t="inlineStr"/>
-      <c r="V19" s="49" t="inlineStr">
+      <c r="V19" s="49" t="inlineStr"/>
+      <c r="W19" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -34107,31 +34167,34 @@
         <v>1344.9</v>
       </c>
       <c r="M20" s="51" t="n">
+        <v>1327.3</v>
+      </c>
+      <c r="N20" s="51" t="n">
         <v>1323.6</v>
       </c>
-      <c r="N20" s="51" t="n">
+      <c r="O20" s="51" t="n">
         <v>1187.13</v>
       </c>
-      <c r="O20" s="51" t="n">
+      <c r="P20" s="51" t="n">
         <v>1176.36</v>
       </c>
-      <c r="P20" s="51" t="n">
+      <c r="Q20" s="51" t="n">
         <v>1166.73</v>
       </c>
-      <c r="Q20" s="51" t="n">
+      <c r="R20" s="51" t="n">
         <v>1100.72</v>
       </c>
-      <c r="R20" s="51" t="n">
+      <c r="S20" s="51" t="n">
         <v>51106.2</v>
       </c>
-      <c r="S20" s="51" t="n">
+      <c r="T20" s="51" t="n">
         <v>737.2</v>
       </c>
-      <c r="T20" s="49" t="n">
+      <c r="U20" s="49" t="n">
         <v>4</v>
       </c>
-      <c r="U20" s="49" t="inlineStr"/>
-      <c r="V20" s="49" t="inlineStr">
+      <c r="V20" s="49" t="inlineStr"/>
+      <c r="W20" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -34185,31 +34248,34 @@
         <v>3092.3</v>
       </c>
       <c r="M21" s="51" t="n">
+        <v>3083.7</v>
+      </c>
+      <c r="N21" s="51" t="n">
         <v>3123.1</v>
       </c>
-      <c r="N21" s="51" t="n">
+      <c r="O21" s="51" t="n">
         <v>3147.77</v>
       </c>
-      <c r="O21" s="51" t="n">
+      <c r="P21" s="51" t="n">
         <v>3151.04</v>
       </c>
-      <c r="P21" s="51" t="n">
+      <c r="Q21" s="51" t="n">
         <v>3153.58</v>
       </c>
-      <c r="Q21" s="51" t="n">
+      <c r="R21" s="51" t="n">
         <v>3162.32</v>
       </c>
-      <c r="R21" s="51" t="n">
+      <c r="S21" s="51" t="n">
         <v>49476.8</v>
       </c>
-      <c r="S21" s="51" t="n">
+      <c r="T21" s="51" t="n">
         <v>-555.2</v>
       </c>
-      <c r="T21" s="49" t="n">
+      <c r="U21" s="49" t="n">
         <v>4</v>
       </c>
-      <c r="U21" s="49" t="inlineStr"/>
-      <c r="V21" s="49" t="inlineStr">
+      <c r="V21" s="49" t="inlineStr"/>
+      <c r="W21" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -34263,31 +34329,34 @@
         <v>78.34</v>
       </c>
       <c r="M22" s="51" t="n">
+        <v>77.8</v>
+      </c>
+      <c r="N22" s="51" t="n">
         <v>78.02</v>
       </c>
-      <c r="N22" s="51" t="n">
+      <c r="O22" s="51" t="n">
         <v>75.51000000000001</v>
       </c>
-      <c r="O22" s="51" t="n">
+      <c r="P22" s="51" t="n">
         <v>74.97</v>
       </c>
-      <c r="P22" s="51" t="n">
+      <c r="Q22" s="51" t="n">
         <v>74.45999999999999</v>
       </c>
-      <c r="Q22" s="51" t="n">
+      <c r="R22" s="51" t="n">
         <v>70.31999999999999</v>
       </c>
-      <c r="R22" s="51" t="n">
+      <c r="S22" s="51" t="n">
         <v>56404.8</v>
       </c>
-      <c r="S22" s="51" t="n">
+      <c r="T22" s="51" t="n">
         <v>1152</v>
       </c>
-      <c r="T22" s="49" t="n">
+      <c r="U22" s="49" t="n">
         <v>123</v>
       </c>
-      <c r="U22" s="49" t="inlineStr"/>
-      <c r="V22" s="49" t="inlineStr">
+      <c r="V22" s="49" t="inlineStr"/>
+      <c r="W22" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -34337,31 +34406,34 @@
         <v>267.61</v>
       </c>
       <c r="M23" s="51" t="n">
+        <v>267.58</v>
+      </c>
+      <c r="N23" s="51" t="n">
         <v>267.3</v>
       </c>
-      <c r="N23" s="51" t="n">
+      <c r="O23" s="51" t="n">
         <v>270.54</v>
       </c>
-      <c r="O23" s="51" t="n">
+      <c r="P23" s="51" t="n">
         <v>270.92</v>
       </c>
-      <c r="P23" s="51" t="n">
+      <c r="Q23" s="51" t="n">
         <v>271.32</v>
       </c>
-      <c r="Q23" s="51" t="n">
+      <c r="R23" s="51" t="n">
         <v>275.06</v>
       </c>
-      <c r="R23" s="51" t="n">
+      <c r="S23" s="51" t="n">
         <v>24620.12</v>
       </c>
-      <c r="S23" s="51" t="n">
+      <c r="T23" s="51" t="n">
         <v>-458.16</v>
       </c>
-      <c r="T23" s="49" t="n">
+      <c r="U23" s="49" t="n">
         <v>71</v>
       </c>
-      <c r="U23" s="49" t="inlineStr"/>
-      <c r="V23" s="49" t="inlineStr">
+      <c r="V23" s="49" t="inlineStr"/>
+      <c r="W23" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -34415,31 +34487,34 @@
         <v>89.02</v>
       </c>
       <c r="M24" s="51" t="n">
+        <v>90.14</v>
+      </c>
+      <c r="N24" s="51" t="n">
         <v>91.41</v>
       </c>
-      <c r="N24" s="51" t="n">
+      <c r="O24" s="51" t="n">
         <v>87.22</v>
       </c>
-      <c r="O24" s="51" t="n">
+      <c r="P24" s="51" t="n">
         <v>86.81</v>
       </c>
-      <c r="P24" s="51" t="n">
+      <c r="Q24" s="51" t="n">
         <v>86.41</v>
       </c>
-      <c r="Q24" s="51" t="n">
+      <c r="R24" s="51" t="n">
         <v>83.20999999999999</v>
       </c>
-      <c r="R24" s="51" t="n">
+      <c r="S24" s="51" t="n">
         <v>26706</v>
       </c>
-      <c r="S24" s="51" t="n">
+      <c r="T24" s="51" t="n">
         <v>1359</v>
       </c>
-      <c r="T24" s="49" t="n">
+      <c r="U24" s="49" t="n">
         <v>137</v>
       </c>
-      <c r="U24" s="49" t="inlineStr"/>
-      <c r="V24" s="49" t="inlineStr">
+      <c r="V24" s="49" t="inlineStr"/>
+      <c r="W24" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -34493,31 +34568,34 @@
         <v>1529.8</v>
       </c>
       <c r="M25" s="51" t="n">
+        <v>1537.5</v>
+      </c>
+      <c r="N25" s="51" t="n">
         <v>1544.8</v>
       </c>
-      <c r="N25" s="51" t="n">
+      <c r="O25" s="51" t="n">
         <v>1355.76</v>
       </c>
-      <c r="O25" s="51" t="n">
+      <c r="P25" s="51" t="n">
         <v>1343.42</v>
       </c>
-      <c r="P25" s="51" t="n">
+      <c r="Q25" s="51" t="n">
         <v>1333.09</v>
       </c>
-      <c r="Q25" s="51" t="n">
+      <c r="R25" s="51" t="n">
         <v>1280.92</v>
       </c>
-      <c r="R25" s="51" t="n">
+      <c r="S25" s="51" t="n">
         <v>107086</v>
       </c>
-      <c r="S25" s="51" t="n">
+      <c r="T25" s="51" t="n">
         <v>7503.3</v>
       </c>
-      <c r="T25" s="49" t="n">
+      <c r="U25" s="49" t="n">
         <v>15</v>
       </c>
-      <c r="U25" s="49" t="inlineStr"/>
-      <c r="V25" s="49" t="inlineStr">
+      <c r="V25" s="49" t="inlineStr"/>
+      <c r="W25" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -34571,31 +34649,34 @@
         <v>9162.5</v>
       </c>
       <c r="M26" s="51" t="n">
+        <v>9151</v>
+      </c>
+      <c r="N26" s="51" t="n">
         <v>9152.5</v>
       </c>
-      <c r="N26" s="51" t="n">
+      <c r="O26" s="51" t="n">
         <v>8992.02</v>
       </c>
-      <c r="O26" s="51" t="n">
+      <c r="P26" s="51" t="n">
         <v>8959.18</v>
       </c>
-      <c r="P26" s="51" t="n">
+      <c r="Q26" s="51" t="n">
         <v>8926.209999999999</v>
       </c>
-      <c r="Q26" s="51" t="n">
+      <c r="R26" s="51" t="n">
         <v>8630.76</v>
       </c>
-      <c r="R26" s="51" t="n">
+      <c r="S26" s="51" t="n">
         <v>458125</v>
       </c>
-      <c r="S26" s="51" t="n">
+      <c r="T26" s="51" t="n">
         <v>71678</v>
       </c>
-      <c r="T26" s="49" t="n">
+      <c r="U26" s="49" t="n">
         <v>253</v>
       </c>
-      <c r="U26" s="49" t="inlineStr"/>
-      <c r="V26" s="49" t="inlineStr">
+      <c r="V26" s="49" t="inlineStr"/>
+      <c r="W26" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -34649,31 +34730,34 @@
         <v>1561.6</v>
       </c>
       <c r="M27" s="51" t="n">
+        <v>1492.1</v>
+      </c>
+      <c r="N27" s="51" t="n">
         <v>1517.8</v>
       </c>
-      <c r="N27" s="51" t="n">
+      <c r="O27" s="51" t="n">
         <v>1499.56</v>
       </c>
-      <c r="O27" s="51" t="n">
+      <c r="P27" s="51" t="n">
         <v>1489.44</v>
       </c>
-      <c r="P27" s="51" t="n">
+      <c r="Q27" s="51" t="n">
         <v>1478.96</v>
       </c>
-      <c r="Q27" s="51" t="n">
+      <c r="R27" s="51" t="n">
         <v>1375.13</v>
       </c>
-      <c r="R27" s="51" t="n">
+      <c r="S27" s="51" t="n">
         <v>65587.2</v>
       </c>
-      <c r="S27" s="51" t="n">
+      <c r="T27" s="51" t="n">
         <v>8724.66</v>
       </c>
-      <c r="T27" s="49" t="n">
+      <c r="U27" s="49" t="n">
         <v>109</v>
       </c>
-      <c r="U27" s="49" t="inlineStr"/>
-      <c r="V27" s="49" t="inlineStr">
+      <c r="V27" s="49" t="inlineStr"/>
+      <c r="W27" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -34727,31 +34811,34 @@
         <v>18116</v>
       </c>
       <c r="M28" s="51" t="n">
+        <v>18019</v>
+      </c>
+      <c r="N28" s="51" t="n">
         <v>17314</v>
       </c>
-      <c r="N28" s="51" t="n">
+      <c r="O28" s="51" t="n">
         <v>16880.24</v>
       </c>
-      <c r="O28" s="51" t="n">
+      <c r="P28" s="51" t="n">
         <v>16786.32</v>
       </c>
-      <c r="P28" s="51" t="n">
+      <c r="Q28" s="51" t="n">
         <v>16699.8</v>
       </c>
-      <c r="Q28" s="51" t="n">
+      <c r="R28" s="51" t="n">
         <v>16053.77</v>
       </c>
-      <c r="R28" s="51" t="n">
+      <c r="S28" s="51" t="n">
         <v>36232</v>
       </c>
-      <c r="S28" s="51" t="n">
+      <c r="T28" s="51" t="n">
         <v>10190</v>
       </c>
-      <c r="T28" s="49" t="n">
+      <c r="U28" s="49" t="n">
         <v>60</v>
       </c>
-      <c r="U28" s="49" t="inlineStr"/>
-      <c r="V28" s="49" t="inlineStr">
+      <c r="V28" s="49" t="inlineStr"/>
+      <c r="W28" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -34805,31 +34892,34 @@
         <v>1882.3</v>
       </c>
       <c r="M29" s="51" t="n">
+        <v>1905.8</v>
+      </c>
+      <c r="N29" s="51" t="n">
         <v>1878.2</v>
       </c>
-      <c r="N29" s="51" t="n">
+      <c r="O29" s="51" t="n">
         <v>1793.32</v>
       </c>
-      <c r="O29" s="51" t="n">
+      <c r="P29" s="51" t="n">
         <v>1787.71</v>
       </c>
-      <c r="P29" s="51" t="n">
+      <c r="Q29" s="51" t="n">
         <v>1782.81</v>
       </c>
-      <c r="Q29" s="51" t="n">
+      <c r="R29" s="51" t="n">
         <v>1753.02</v>
       </c>
-      <c r="R29" s="51" t="n">
+      <c r="S29" s="51" t="n">
         <v>48939.8</v>
       </c>
-      <c r="S29" s="51" t="n">
+      <c r="T29" s="51" t="n">
         <v>-439.4</v>
       </c>
-      <c r="T29" s="49" t="n">
+      <c r="U29" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="U29" s="49" t="inlineStr"/>
-      <c r="V29" s="49" t="inlineStr">
+      <c r="V29" s="49" t="inlineStr"/>
+      <c r="W29" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -34883,31 +34973,34 @@
         <v>1256.3</v>
       </c>
       <c r="M30" s="51" t="n">
+        <v>1328</v>
+      </c>
+      <c r="N30" s="51" t="n">
         <v>1311.3</v>
       </c>
-      <c r="N30" s="51" t="n">
+      <c r="O30" s="51" t="n">
         <v>1232.7</v>
       </c>
-      <c r="O30" s="51" t="n">
+      <c r="P30" s="51" t="n">
         <v>1226.66</v>
       </c>
-      <c r="P30" s="51" t="n">
+      <c r="Q30" s="51" t="n">
         <v>1220.66</v>
       </c>
-      <c r="Q30" s="51" t="n">
+      <c r="R30" s="51" t="n">
         <v>1162.77</v>
       </c>
-      <c r="R30" s="51" t="n">
+      <c r="S30" s="51" t="n">
         <v>371864.8</v>
       </c>
-      <c r="S30" s="51" t="n">
+      <c r="T30" s="51" t="n">
         <v>97090.96000000001</v>
       </c>
-      <c r="T30" s="49" t="n">
+      <c r="U30" s="49" t="n">
         <v>96</v>
       </c>
-      <c r="U30" s="49" t="inlineStr"/>
-      <c r="V30" s="49" t="inlineStr">
+      <c r="V30" s="49" t="inlineStr"/>
+      <c r="W30" s="49" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
feat: add conditional formatting for Prev_Day_Close and Prev_Week_Close columns in Excel and Google Sheets
</commit_message>
<xml_diff>
--- a/Transformed_Tradebook.xlsx
+++ b/Transformed_Tradebook.xlsx
@@ -127,7 +127,7 @@
       <color rgb="00C00000"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -144,6 +144,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="002F5496"/>
         <bgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+        <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+        <bgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -239,7 +251,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -310,6 +322,8 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="5" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -32704,10 +32718,10 @@
       <c r="L2" s="51" t="n">
         <v>2886.5</v>
       </c>
-      <c r="M2" s="51" t="n">
+      <c r="M2" s="54" t="n">
         <v>2799.1</v>
       </c>
-      <c r="N2" s="51" t="n">
+      <c r="N2" s="54" t="n">
         <v>2731</v>
       </c>
       <c r="O2" s="51" t="n">
@@ -32785,10 +32799,10 @@
       <c r="L3" s="51" t="n">
         <v>2725</v>
       </c>
-      <c r="M3" s="51" t="n">
+      <c r="M3" s="54" t="n">
         <v>2689.8</v>
       </c>
-      <c r="N3" s="51" t="n">
+      <c r="N3" s="54" t="n">
         <v>2716</v>
       </c>
       <c r="O3" s="51" t="n">
@@ -32866,10 +32880,10 @@
       <c r="L4" s="51" t="n">
         <v>3248.2</v>
       </c>
-      <c r="M4" s="51" t="n">
+      <c r="M4" s="54" t="n">
         <v>3214.1</v>
       </c>
-      <c r="N4" s="51" t="n">
+      <c r="N4" s="54" t="n">
         <v>3177.2</v>
       </c>
       <c r="O4" s="51" t="n">
@@ -32947,10 +32961,10 @@
       <c r="L5" s="51" t="n">
         <v>1864.5</v>
       </c>
-      <c r="M5" s="51" t="n">
+      <c r="M5" s="55" t="n">
         <v>1876</v>
       </c>
-      <c r="N5" s="51" t="n">
+      <c r="N5" s="55" t="n">
         <v>1890.2</v>
       </c>
       <c r="O5" s="51" t="n">
@@ -33028,10 +33042,10 @@
       <c r="L6" s="51" t="n">
         <v>340.7</v>
       </c>
-      <c r="M6" s="51" t="n">
+      <c r="M6" s="54" t="n">
         <v>311</v>
       </c>
-      <c r="N6" s="51" t="n">
+      <c r="N6" s="54" t="n">
         <v>294.55</v>
       </c>
       <c r="O6" s="51" t="n">
@@ -33109,10 +33123,10 @@
       <c r="L7" s="51" t="n">
         <v>1092.7</v>
       </c>
-      <c r="M7" s="51" t="n">
+      <c r="M7" s="54" t="n">
         <v>1087.2</v>
       </c>
-      <c r="N7" s="51" t="n">
+      <c r="N7" s="55" t="n">
         <v>1106.6</v>
       </c>
       <c r="O7" s="51" t="n">
@@ -33190,10 +33204,10 @@
       <c r="L8" s="51" t="n">
         <v>1512.8</v>
       </c>
-      <c r="M8" s="51" t="n">
+      <c r="M8" s="54" t="n">
         <v>1500.5</v>
       </c>
-      <c r="N8" s="51" t="n">
+      <c r="N8" s="54" t="n">
         <v>1511.8</v>
       </c>
       <c r="O8" s="51" t="n">
@@ -33271,10 +33285,10 @@
       <c r="L9" s="51" t="n">
         <v>1708.8</v>
       </c>
-      <c r="M9" s="51" t="n">
+      <c r="M9" s="55" t="n">
         <v>1763</v>
       </c>
-      <c r="N9" s="51" t="n">
+      <c r="N9" s="54" t="n">
         <v>1706.2</v>
       </c>
       <c r="O9" s="51" t="n">
@@ -33352,10 +33366,10 @@
       <c r="L10" s="51" t="n">
         <v>4190.8</v>
       </c>
-      <c r="M10" s="51" t="n">
+      <c r="M10" s="54" t="n">
         <v>4120.7</v>
       </c>
-      <c r="N10" s="51" t="n">
+      <c r="N10" s="54" t="n">
         <v>4000.6</v>
       </c>
       <c r="O10" s="51" t="n">
@@ -33433,10 +33447,10 @@
       <c r="L11" s="51" t="n">
         <v>1089.4</v>
       </c>
-      <c r="M11" s="51" t="n">
+      <c r="M11" s="55" t="n">
         <v>1090.4</v>
       </c>
-      <c r="N11" s="51" t="n">
+      <c r="N11" s="55" t="n">
         <v>1116.3</v>
       </c>
       <c r="O11" s="51" t="n">
@@ -33514,10 +33528,10 @@
       <c r="L12" s="51" t="n">
         <v>819.4</v>
       </c>
-      <c r="M12" s="51" t="n">
+      <c r="M12" s="54" t="n">
         <v>808.75</v>
       </c>
-      <c r="N12" s="51" t="n">
+      <c r="N12" s="55" t="n">
         <v>838.2</v>
       </c>
       <c r="O12" s="51" t="n">
@@ -33595,10 +33609,10 @@
       <c r="L13" s="51" t="n">
         <v>114.34</v>
       </c>
-      <c r="M13" s="51" t="n">
+      <c r="M13" s="55" t="n">
         <v>120.84</v>
       </c>
-      <c r="N13" s="51" t="n">
+      <c r="N13" s="55" t="n">
         <v>120.36</v>
       </c>
       <c r="O13" s="51" t="n">
@@ -33680,10 +33694,10 @@
       <c r="L14" s="51" t="n">
         <v>286.6</v>
       </c>
-      <c r="M14" s="51" t="n">
+      <c r="M14" s="54" t="n">
         <v>283.95</v>
       </c>
-      <c r="N14" s="51" t="n">
+      <c r="N14" s="54" t="n">
         <v>281.3</v>
       </c>
       <c r="O14" s="51" t="n">
@@ -33761,10 +33775,10 @@
       <c r="L15" s="51" t="n">
         <v>161.12</v>
       </c>
-      <c r="M15" s="51" t="n">
+      <c r="M15" s="55" t="n">
         <v>161.98</v>
       </c>
-      <c r="N15" s="51" t="n">
+      <c r="N15" s="55" t="n">
         <v>162.79</v>
       </c>
       <c r="O15" s="51" t="n">
@@ -33842,10 +33856,10 @@
       <c r="L16" s="51" t="n">
         <v>643.85</v>
       </c>
-      <c r="M16" s="51" t="n">
+      <c r="M16" s="54" t="n">
         <v>632.8</v>
       </c>
-      <c r="N16" s="51" t="n">
+      <c r="N16" s="55" t="n">
         <v>652.6</v>
       </c>
       <c r="O16" s="51" t="n">
@@ -33923,10 +33937,10 @@
       <c r="L17" s="51" t="n">
         <v>290.55</v>
       </c>
-      <c r="M17" s="51" t="n">
+      <c r="M17" s="54" t="n">
         <v>283.3</v>
       </c>
-      <c r="N17" s="51" t="n">
+      <c r="N17" s="54" t="n">
         <v>287.9</v>
       </c>
       <c r="O17" s="51" t="n">
@@ -34004,10 +34018,10 @@
       <c r="L18" s="51" t="n">
         <v>4385.3</v>
       </c>
-      <c r="M18" s="51" t="n">
+      <c r="M18" s="55" t="n">
         <v>4426.8</v>
       </c>
-      <c r="N18" s="51" t="n">
+      <c r="N18" s="54" t="n">
         <v>4342.6</v>
       </c>
       <c r="O18" s="51" t="n">
@@ -34085,10 +34099,10 @@
       <c r="L19" s="51" t="n">
         <v>1048.3</v>
       </c>
-      <c r="M19" s="51" t="n">
+      <c r="M19" s="55" t="n">
         <v>1053.1</v>
       </c>
-      <c r="N19" s="51" t="n">
+      <c r="N19" s="55" t="n">
         <v>1067.5</v>
       </c>
       <c r="O19" s="51" t="n">
@@ -34166,10 +34180,10 @@
       <c r="L20" s="51" t="n">
         <v>1344.9</v>
       </c>
-      <c r="M20" s="51" t="n">
+      <c r="M20" s="54" t="n">
         <v>1327.3</v>
       </c>
-      <c r="N20" s="51" t="n">
+      <c r="N20" s="54" t="n">
         <v>1323.6</v>
       </c>
       <c r="O20" s="51" t="n">
@@ -34247,10 +34261,10 @@
       <c r="L21" s="51" t="n">
         <v>3092.3</v>
       </c>
-      <c r="M21" s="51" t="n">
+      <c r="M21" s="54" t="n">
         <v>3083.7</v>
       </c>
-      <c r="N21" s="51" t="n">
+      <c r="N21" s="55" t="n">
         <v>3123.1</v>
       </c>
       <c r="O21" s="51" t="n">
@@ -34328,10 +34342,10 @@
       <c r="L22" s="51" t="n">
         <v>78.34</v>
       </c>
-      <c r="M22" s="51" t="n">
+      <c r="M22" s="54" t="n">
         <v>77.8</v>
       </c>
-      <c r="N22" s="51" t="n">
+      <c r="N22" s="54" t="n">
         <v>78.02</v>
       </c>
       <c r="O22" s="51" t="n">
@@ -34405,10 +34419,10 @@
       <c r="L23" s="51" t="n">
         <v>267.61</v>
       </c>
-      <c r="M23" s="51" t="n">
+      <c r="M23" s="54" t="n">
         <v>267.58</v>
       </c>
-      <c r="N23" s="51" t="n">
+      <c r="N23" s="54" t="n">
         <v>267.3</v>
       </c>
       <c r="O23" s="51" t="n">
@@ -34486,10 +34500,10 @@
       <c r="L24" s="51" t="n">
         <v>89.02</v>
       </c>
-      <c r="M24" s="51" t="n">
+      <c r="M24" s="55" t="n">
         <v>90.14</v>
       </c>
-      <c r="N24" s="51" t="n">
+      <c r="N24" s="55" t="n">
         <v>91.41</v>
       </c>
       <c r="O24" s="51" t="n">
@@ -34567,10 +34581,10 @@
       <c r="L25" s="51" t="n">
         <v>1529.8</v>
       </c>
-      <c r="M25" s="51" t="n">
+      <c r="M25" s="55" t="n">
         <v>1537.5</v>
       </c>
-      <c r="N25" s="51" t="n">
+      <c r="N25" s="55" t="n">
         <v>1544.8</v>
       </c>
       <c r="O25" s="51" t="n">
@@ -34648,10 +34662,10 @@
       <c r="L26" s="51" t="n">
         <v>9162.5</v>
       </c>
-      <c r="M26" s="51" t="n">
+      <c r="M26" s="54" t="n">
         <v>9151</v>
       </c>
-      <c r="N26" s="51" t="n">
+      <c r="N26" s="54" t="n">
         <v>9152.5</v>
       </c>
       <c r="O26" s="51" t="n">
@@ -34729,10 +34743,10 @@
       <c r="L27" s="51" t="n">
         <v>1561.6</v>
       </c>
-      <c r="M27" s="51" t="n">
+      <c r="M27" s="54" t="n">
         <v>1492.1</v>
       </c>
-      <c r="N27" s="51" t="n">
+      <c r="N27" s="54" t="n">
         <v>1517.8</v>
       </c>
       <c r="O27" s="51" t="n">
@@ -34810,10 +34824,10 @@
       <c r="L28" s="51" t="n">
         <v>18116</v>
       </c>
-      <c r="M28" s="51" t="n">
+      <c r="M28" s="54" t="n">
         <v>18019</v>
       </c>
-      <c r="N28" s="51" t="n">
+      <c r="N28" s="54" t="n">
         <v>17314</v>
       </c>
       <c r="O28" s="51" t="n">
@@ -34891,10 +34905,10 @@
       <c r="L29" s="51" t="n">
         <v>1882.3</v>
       </c>
-      <c r="M29" s="51" t="n">
+      <c r="M29" s="55" t="n">
         <v>1905.8</v>
       </c>
-      <c r="N29" s="51" t="n">
+      <c r="N29" s="54" t="n">
         <v>1878.2</v>
       </c>
       <c r="O29" s="51" t="n">
@@ -34972,10 +34986,10 @@
       <c r="L30" s="51" t="n">
         <v>1256.3</v>
       </c>
-      <c r="M30" s="51" t="n">
+      <c r="M30" s="55" t="n">
         <v>1328</v>
       </c>
-      <c r="N30" s="51" t="n">
+      <c r="N30" s="55" t="n">
         <v>1311.3</v>
       </c>
       <c r="O30" s="51" t="n">

</xml_diff>